<commit_message>
updated species names to merge
</commit_message>
<xml_diff>
--- a/annotation/Species_list_2022_10_06.xlsx
+++ b/annotation/Species_list_2022_10_06.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jjansen\Desktop\science\SouthernOceanBiodiversityMapping\ARC_Data\annotation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56231F09-99F6-41A6-B503-4A0378D56263}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD38F59E-9529-4484-A043-1DF4F99BB2BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15030" yWindow="-18120" windowWidth="29040" windowHeight="18240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-13770" yWindow="-18120" windowWidth="29040" windowHeight="18240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="COVER_prevalence" sheetId="1" r:id="rId1"/>
@@ -2444,7 +2444,7 @@
         <v>1.9E-2</v>
       </c>
       <c r="F97" t="s">
-        <v>247</v>
+        <v>18</v>
       </c>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.3">

</xml_diff>